<commit_message>
fix(report): rho_pf as prefill load C_model*SL_pf_eff/Th_pf (methodology 6.2)
Co-authored-by: Perplexity Computer <computer@perplexity.ai>
</commit_message>
<xml_diff>
--- a/backend/reportTemplate.xlsx
+++ b/backend/reportTemplate.xlsx
@@ -5204,12 +5204,12 @@
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>ρ_pf (доля времени prefill, диагностика §6.2)</t>
+          <t>ρ_pf (загрузка prefill, диагностика §6.2)</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>(SL_pf^eff/Th_pf) / (SL_pf^eff/Th_pf + T_dec/Th_dec) при BS итоговом</t>
+          <t>C^model · SL_pf^eff / Th_pf — среднее число запросов в prefill; &gt; 1 → prefill в очереди, C^model завышен (проверить нагрузочным тестом / PD)</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -5218,7 +5218,7 @@
         </is>
       </c>
       <c r="D57" s="30">
-        <f>IF(AND(D33&gt;0,D38&gt;0),(D27/D33)/(D27/D33+Inputs!D22/D38),0)</f>
+        <f>IF(D33&gt;0,D39*D27/D33,0)</f>
         <v/>
       </c>
       <c r="E57" s="4" t="inlineStr">

</xml_diff>